<commit_message>
feat(viceri-study): publish specification and test suite v1.4
</commit_message>
<xml_diff>
--- a/output/xlsx/AdministradorAdicionaEcommerce--GT-.xlsx
+++ b/output/xlsx/AdministradorAdicionaEcommerce--GT-.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="56">
   <si>
     <t xml:space="preserve">System: </t>
   </si>
@@ -38,7 +38,7 @@
     <t>Reduced (Greedy Heuristic - Transition Coverage)</t>
   </si>
   <si>
-    <t>Size: 5 test case(s)</t>
+    <t>Size: 6 test case(s)</t>
   </si>
   <si>
     <t xml:space="preserve">Creation Date: </t>
@@ -101,7 +101,7 @@
     <t>SYSTEM exibe tela inicial do sistema</t>
   </si>
   <si>
-    <t>Administrador: clica no opcao 'Ecommerces' no menu principal</t>
+    <t>Administrador: clica no opcao 'E-commerces' no menu principal</t>
   </si>
   <si>
     <t>SYSTEM exibe a tela com a lista de E-commerces cadastrados no sistema</t>
@@ -122,7 +122,7 @@
     <t xml:space="preserve">Postcondition: </t>
   </si>
   <si>
-    <t>O novo E-commerce esta salvo no sistema.</t>
+    <t>O novo E-commerce salvo no sistema.</t>
   </si>
   <si>
     <t>TC2</t>
@@ -131,7 +131,7 @@
     <t>Alternative Flow 1: Volta para tela inicial do sistema</t>
   </si>
   <si>
-    <t>Administrador: clica no botao 'Voltar'</t>
+    <t>Administrador: clica no botao Voltar</t>
   </si>
   <si>
     <t>TC3</t>
@@ -140,13 +140,22 @@
     <t>Alternative Flow 2: Cancela registro de Ecommerce</t>
   </si>
   <si>
-    <t>Administrador: clica no botao 'Cancelar'</t>
+    <t>Administrador: clica no botao Cancelar</t>
   </si>
   <si>
     <t>TC4</t>
   </si>
   <si>
-    <t>Exception Flow 1: Nao preenche algum campo obrigatorio</t>
+    <t>Alternative Flow 3: Navega pela lista de Ecommerce</t>
+  </si>
+  <si>
+    <t>Administrador: clica no botao de paginacao</t>
+  </si>
+  <si>
+    <t>TC5</t>
+  </si>
+  <si>
+    <t>Exception Flow 1: Nao preencher campos obrigatorios</t>
   </si>
   <si>
     <t>SYSTEM alerta ao usuario que os campos obrigatorios devem ser preenchidos</t>
@@ -161,7 +170,7 @@
     <t>Flow interrupted due to exception / error</t>
   </si>
   <si>
-    <t>TC5</t>
+    <t>TC6</t>
   </si>
   <si>
     <t>Exception Flow 2: Conflito de CNPJ</t>
@@ -262,7 +271,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
@@ -873,13 +882,13 @@
         <v>1.0</v>
       </c>
       <c r="B47" t="s" s="3">
-        <v>26</v>
+        <v>45</v>
       </c>
       <c r="C47" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D47" t="s" s="3">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E47" t="s" s="3">
         <v>27</v>
@@ -893,13 +902,13 @@
         <v>2.0</v>
       </c>
       <c r="B48" t="s" s="3">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C48" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D48" t="s" s="3">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E48" t="s" s="3">
         <v>27</v>
@@ -913,13 +922,13 @@
         <v>3.0</v>
       </c>
       <c r="B49" t="s" s="3">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C49" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D49" t="s" s="3">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E49" t="s" s="3">
         <v>27</v>
@@ -929,118 +938,118 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="n" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="B50" t="s" s="3">
-        <v>33</v>
-      </c>
-      <c r="C50" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D50" t="s" s="3">
-        <v>45</v>
-      </c>
-      <c r="E50" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F50" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="B51" t="s" s="3">
+      <c r="A50" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="B50" t="s" s="0">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B53" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="C51" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D51" t="s" s="3">
+      <c r="C53" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E53" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B54" t="s" s="0">
         <v>47</v>
       </c>
-      <c r="E51" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F51" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="B52" t="s" s="0">
-        <v>48</v>
+      <c r="E54" t="s" s="1">
+        <v>17</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="1">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>49</v>
-      </c>
-      <c r="C55" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E55" t="s" s="1">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="B56" t="s" s="0">
-        <v>50</v>
-      </c>
-      <c r="E56" t="s" s="1">
-        <v>17</v>
+      <c r="A56" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B56" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C56" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D56" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E56" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F56" t="s" s="2">
+        <v>25</v>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="s" s="1">
-        <v>18</v>
-      </c>
-      <c r="B57" t="s" s="0">
-        <v>19</v>
+      <c r="A57" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B57" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C57" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D57" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E57" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F57" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="s" s="2">
-        <v>20</v>
-      </c>
-      <c r="B58" t="s" s="2">
-        <v>21</v>
-      </c>
-      <c r="C58" t="s" s="2">
-        <v>22</v>
-      </c>
-      <c r="D58" t="s" s="2">
-        <v>23</v>
-      </c>
-      <c r="E58" t="s" s="2">
-        <v>24</v>
-      </c>
-      <c r="F58" t="s" s="2">
-        <v>25</v>
+      <c r="A58" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B58" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C58" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D58" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E58" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F58" t="s" s="3">
+        <v>27</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n" s="4">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="B59" t="s" s="3">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C59" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D59" t="s" s="3">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E59" t="s" s="3">
         <v>27</v>
@@ -1051,16 +1060,16 @@
     </row>
     <row r="60">
       <c r="A60" t="n" s="4">
-        <v>2.0</v>
+        <v>4.0</v>
       </c>
       <c r="B60" t="s" s="3">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C60" t="s" s="3">
         <v>27</v>
       </c>
       <c r="D60" t="s" s="3">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="E60" t="s" s="3">
         <v>27</v>
@@ -1071,70 +1080,191 @@
     </row>
     <row r="61">
       <c r="A61" t="n" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B61" t="s" s="3">
+        <v>49</v>
+      </c>
+      <c r="C61" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D61" t="s" s="3">
+        <v>50</v>
+      </c>
+      <c r="E61" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F61" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="B62" t="s" s="0">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="B65" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="C65" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E65" t="s" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="B66" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="E66" t="s" s="1">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s" s="1">
+        <v>18</v>
+      </c>
+      <c r="B67" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s" s="2">
+        <v>20</v>
+      </c>
+      <c r="B68" t="s" s="2">
+        <v>21</v>
+      </c>
+      <c r="C68" t="s" s="2">
+        <v>22</v>
+      </c>
+      <c r="D68" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="E68" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="F68" t="s" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B69" t="s" s="3">
+        <v>26</v>
+      </c>
+      <c r="C69" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D69" t="s" s="3">
+        <v>28</v>
+      </c>
+      <c r="E69" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F69" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B70" t="s" s="3">
+        <v>29</v>
+      </c>
+      <c r="C70" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D70" t="s" s="3">
+        <v>30</v>
+      </c>
+      <c r="E70" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F70" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n" s="4">
         <v>3.0</v>
       </c>
-      <c r="B61" t="s" s="3">
+      <c r="B71" t="s" s="3">
         <v>31</v>
       </c>
-      <c r="C61" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D61" t="s" s="3">
+      <c r="C71" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D71" t="s" s="3">
         <v>32</v>
       </c>
-      <c r="E61" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F61" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="n" s="4">
+      <c r="E71" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F71" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n" s="4">
         <v>4.0</v>
       </c>
-      <c r="B62" t="s" s="3">
+      <c r="B72" t="s" s="3">
         <v>33</v>
       </c>
-      <c r="C62" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D62" t="s" s="3">
+      <c r="C72" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D72" t="s" s="3">
+        <v>54</v>
+      </c>
+      <c r="E72" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F72" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B73" t="s" s="3">
+        <v>55</v>
+      </c>
+      <c r="C73" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="D73" t="s" s="3">
+        <v>50</v>
+      </c>
+      <c r="E73" t="s" s="3">
+        <v>27</v>
+      </c>
+      <c r="F73" t="s" s="3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="B74" t="s" s="0">
         <v>51</v>
-      </c>
-      <c r="E62" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F62" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="n" s="4">
-        <v>5.0</v>
-      </c>
-      <c r="B63" t="s" s="3">
-        <v>52</v>
-      </c>
-      <c r="C63" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="D63" t="s" s="3">
-        <v>47</v>
-      </c>
-      <c r="E63" t="s" s="3">
-        <v>27</v>
-      </c>
-      <c r="F63" t="s" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="B64" t="s" s="0">
-        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>